<commit_message>
Add timestamp functionality to Master Aggregator
- CSV files now include timestamps in filenames (YYYYMMDD_HHMM format)
- Excel Methodology sheet includes 'Last Updated' field
- Enables tracking multiple analysis runs over time
- Updated README to mark timestamp feature as completed
</commit_message>
<xml_diff>
--- a/master_investment_rankings.xlsx
+++ b/master_investment_rankings.xlsx
@@ -47701,7 +47701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -47988,6 +47988,22 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Last Updated: 2026-05-31 16:54</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add sector-adjusted rankings feature
- Calculate rankings within each sector for better comparison
- New 'Best Per Sector' Excel sheet showing top stock in each sector
- Console output displays best stock per sector with overall and sector ranks
- Sector-specific percentile rankings for relative performance
- Helps identify sector leaders and diversification opportunities
- Updated README to mark feature as completed
</commit_message>
<xml_diff>
--- a/master_investment_rankings.xlsx
+++ b/master_investment_rankings.xlsx
@@ -11,7 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Rankings" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grade A Stocks" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grade B Stocks" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Best Per Sector" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47701,6 +47702,512 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Composite_Score</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Investment_Grade</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Percentile</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Sector_Rank</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Sector_Percentile</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Average_Rank</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Tools_Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>INCY</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Incyte Corporation</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>A+ (Exceptional)</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1.851851851851852</v>
+      </c>
+      <c r="I2" t="n">
+        <v>41</v>
+      </c>
+      <c r="J2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>APA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>APA Corporation</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>A+ (Exceptional)</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>99.78902953586498</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>4.761904761904762</v>
+      </c>
+      <c r="I3" t="n">
+        <v>42.25</v>
+      </c>
+      <c r="J3" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Altria Group, Inc.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Consumer Defensive</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>A+ (Exceptional)</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>99.57805907172997</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>3.448275862068965</v>
+      </c>
+      <c r="I4" t="n">
+        <v>46.33333333333334</v>
+      </c>
+      <c r="J4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>HPQ</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HP Inc.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>A+ (Exceptional)</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>99.36708860759494</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="I5" t="n">
+        <v>56</v>
+      </c>
+      <c r="J5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Lowe's Companies, Inc.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>A+ (Exceptional)</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>99.15611814345992</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" t="n">
+        <v>65</v>
+      </c>
+      <c r="J6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SYF</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Synchrony Financial</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>A+ (Exceptional)</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>98.73417721518987</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1.470588235294118</v>
+      </c>
+      <c r="I7" t="n">
+        <v>73.85714285714286</v>
+      </c>
+      <c r="J7" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CHTR</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Charter Communications, Inc.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>A+ (Exceptional)</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>98.52320675105484</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>5.263157894736842</v>
+      </c>
+      <c r="I8" t="n">
+        <v>74.85714285714286</v>
+      </c>
+      <c r="J8" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MAS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Masco Corporation</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>16</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>A+ (Exceptional)</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>96.83544303797468</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1.351351351351351</v>
+      </c>
+      <c r="I9" t="n">
+        <v>85.16666666666667</v>
+      </c>
+      <c r="J9" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CF Industries Holdings, Inc.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Basic Materials</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>18</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>A+ (Exceptional)</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>96.41350210970464</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" t="n">
+        <v>5.88235294117647</v>
+      </c>
+      <c r="I10" t="n">
+        <v>87.75</v>
+      </c>
+      <c r="J10" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>EIX</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Edison International</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>21</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>A+ (Exceptional)</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>95.78059071729957</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>3.225806451612903</v>
+      </c>
+      <c r="I11" t="n">
+        <v>91.57142857142857</v>
+      </c>
+      <c r="J11" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>IRM</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Iron Mountain Incorporated</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>62</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>A (Excellent)</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>87.13080168776372</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3.333333333333333</v>
+      </c>
+      <c r="I12" t="n">
+        <v>123</v>
+      </c>
+      <c r="J12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -48000,7 +48507,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Last Updated: 2026-05-31 16:54</t>
+          <t>Last Updated: 2026-05-31 17:05</t>
         </is>
       </c>
     </row>

</xml_diff>